<commit_message>
feat: add import rollback audit trail
</commit_message>
<xml_diff>
--- a/storage/app/private/kompen-respon-hub/Template_Impor_Kompen_Respon_Hub.xlsx
+++ b/storage/app/private/kompen-respon-hub/Template_Impor_Kompen_Respon_Hub.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="1" r:id="R998ce8ad492a4b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kompen dan Respon" sheetId="2" r:id="R9f29b55617f34926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail Kompen" sheetId="3" r:id="Rba5b1ec5bc674632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="1" r:id="R794a44fb3c2b40cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kompen dan Respon" sheetId="2" r:id="R19c00ff326f1498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail Kompen" sheetId="3" r:id="Rd0ff518747bd4312"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44234,70 +44234,54 @@
       <x:c r="AY679" s="149" t="str"/>
     </x:row>
     <x:row r="680">
-      <x:c r="A680" s="38" t="str">
-        <x:f>IF(B680="","",COUNTIF($B$646:B680,"&lt;&gt;"))</x:f>
-      </x:c>
-      <x:c r="B680" s="40" t="str"/>
-      <x:c r="C680" s="15" t="str"/>
-      <x:c r="D680" s="41" t="str"/>
-      <x:c r="E680" s="41" t="str"/>
-      <x:c r="F680" s="41" t="str"/>
-      <x:c r="G680" s="41" t="str"/>
-      <x:c r="H680" s="41" t="str"/>
-      <x:c r="I680" s="41" t="str"/>
-      <x:c r="J680" s="42" t="str">
-        <x:f>IF(B680="","",H680+I680)</x:f>
-      </x:c>
-      <x:c r="K680" s="42" t="str"/>
-      <x:c r="L680" s="42" t="str"/>
-      <x:c r="N680" s="38" t="str">
-        <x:f>IF(O680="","",COUNTIF($O$646:O680,"&lt;&gt;"))</x:f>
-      </x:c>
-      <x:c r="O680" s="40" t="str"/>
-      <x:c r="P680" s="15" t="str"/>
-      <x:c r="Q680" s="41" t="str"/>
-      <x:c r="R680" s="41" t="str"/>
-      <x:c r="S680" s="41" t="str"/>
-      <x:c r="T680" s="41" t="str"/>
-      <x:c r="U680" s="41" t="str"/>
-      <x:c r="V680" s="41" t="str"/>
-      <x:c r="W680" s="42" t="str">
-        <x:f>IF(O680="","",U680+V680)</x:f>
-      </x:c>
-      <x:c r="X680" s="42" t="str"/>
-      <x:c r="Y680" s="42" t="str"/>
-      <x:c r="AA680" s="38" t="str">
-        <x:f>IF(AB680="","",COUNTIF($AB$646:AB680,"&lt;&gt;"))</x:f>
-      </x:c>
-      <x:c r="AB680" s="40" t="str"/>
-      <x:c r="AC680" s="15" t="str"/>
-      <x:c r="AD680" s="41" t="str"/>
-      <x:c r="AE680" s="41" t="str"/>
-      <x:c r="AF680" s="41" t="str"/>
-      <x:c r="AG680" s="41" t="str"/>
-      <x:c r="AH680" s="41" t="str"/>
-      <x:c r="AI680" s="41" t="str"/>
-      <x:c r="AJ680" s="42" t="str">
-        <x:f>IF(AB680="","",AH680+AI680)</x:f>
-      </x:c>
-      <x:c r="AK680" s="42" t="str"/>
-      <x:c r="AL680" s="42" t="str"/>
-      <x:c r="AN680" s="38" t="str">
-        <x:f>IF(AO680="","",COUNTIF($AO$646:AO680,"&lt;&gt;"))</x:f>
-      </x:c>
-      <x:c r="AO680" s="40" t="str"/>
-      <x:c r="AP680" s="15" t="str"/>
-      <x:c r="AQ680" s="41" t="str"/>
-      <x:c r="AR680" s="41" t="str"/>
-      <x:c r="AS680" s="41" t="str"/>
-      <x:c r="AT680" s="41" t="str"/>
-      <x:c r="AU680" s="41" t="str"/>
-      <x:c r="AV680" s="41" t="str"/>
-      <x:c r="AW680" s="42" t="str">
-        <x:f>IF(AO680="","",AU680+AV680)</x:f>
-      </x:c>
-      <x:c r="AX680" s="42" t="str"/>
-      <x:c r="AY680" s="42" t="str"/>
+      <x:c r="A680"/>
+      <x:c r="B680"/>
+      <x:c r="C680"/>
+      <x:c r="D680"/>
+      <x:c r="E680"/>
+      <x:c r="F680"/>
+      <x:c r="G680"/>
+      <x:c r="H680"/>
+      <x:c r="I680"/>
+      <x:c r="J680"/>
+      <x:c r="K680"/>
+      <x:c r="L680"/>
+      <x:c r="N680"/>
+      <x:c r="O680"/>
+      <x:c r="P680"/>
+      <x:c r="Q680"/>
+      <x:c r="R680"/>
+      <x:c r="S680"/>
+      <x:c r="T680"/>
+      <x:c r="U680"/>
+      <x:c r="V680"/>
+      <x:c r="W680"/>
+      <x:c r="X680"/>
+      <x:c r="Y680"/>
+      <x:c r="AA680"/>
+      <x:c r="AB680"/>
+      <x:c r="AC680"/>
+      <x:c r="AD680"/>
+      <x:c r="AE680"/>
+      <x:c r="AF680"/>
+      <x:c r="AG680"/>
+      <x:c r="AH680"/>
+      <x:c r="AI680"/>
+      <x:c r="AJ680"/>
+      <x:c r="AK680"/>
+      <x:c r="AL680"/>
+      <x:c r="AN680"/>
+      <x:c r="AO680"/>
+      <x:c r="AP680"/>
+      <x:c r="AQ680"/>
+      <x:c r="AR680"/>
+      <x:c r="AS680"/>
+      <x:c r="AT680"/>
+      <x:c r="AU680"/>
+      <x:c r="AV680"/>
+      <x:c r="AW680"/>
+      <x:c r="AX680"/>
+      <x:c r="AY680"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>